<commit_message>
fix(tr-109): actually add TR-Juan-109 to KB v1.9 (bug: --confidence enum required HIGH not 7)
- kb_editor add-rule had failed silently in previous run (passed --confidence 7, requires HIGH/MEDIUM/LOW/MAXIMA)
- Resultado: v1.9 era idéntica a v1.8, sin TR-109. PnL comparison reportó 0 diff porque ambos engines tenían misma KB.
- También: deploy.spike.sh ahora pasa --set-secrets para ANTHROPIC_API_KEY (engine C había caído por env var faltante)
</commit_message>
<xml_diff>
--- a/llm_engine_eolo/kb/EOLO_ThetaHarvest_v1.9.xlsx
+++ b/llm_engine_eolo/kb/EOLO_ThetaHarvest_v1.9.xlsx
@@ -4463,7 +4463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I109"/>
+  <dimension ref="A1:I110"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="33" min="1" max="1"/>
@@ -4898,7 +4898,7 @@
           <t>PROHIBITIVA</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I10" s="33" t="inlineStr">
         <is>
           <t>TR-Juan-083</t>
         </is>
@@ -8813,6 +8813,44 @@
       </c>
       <c r="G109" s="33" t="inlineStr"/>
       <c r="H109" s="33" t="inlineStr">
+        <is>
+          <t>MAESTRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>TR-Juan-109</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>VIX_SPIKE_DIRECTIONAL_BIAS</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Cuando vix_velocity_30m_pct &gt; +5% Y price_change_30m &lt; -0.5%: PREFERIR SELL_CALL_SPREAD direccional. Cushion ASIMÉTRICO (CALL cushion×2, PUT cushion×1). Strike CALL en ema21_daily o resistencia local. DTE 0-2. Confidence HIGH. Sizing baseline. NO IC en este régimen. INVERSO: vix_velocity &lt; -5% Y price_change &gt; +0.5% -&gt; PREFERIR SELL_PUT_SPREAD.</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Captura asimetría VIX/precio durante spikes. NO se aplica si vix_velocity &lt; +5%. Validada con eventos históricos.</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
         <is>
           <t>MAESTRA</t>
         </is>

</xml_diff>